<commit_message>
fix(eval): reframe benchmark as controlled pilot micro-benchmark (N=12) with explicit threats to validity
</commit_message>
<xml_diff>
--- a/Literature_Review_Member_Assignments.xlsx
+++ b/Literature_Review_Member_Assignments.xlsx
@@ -2506,7 +2506,7 @@
     <row r="19" ht="65" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Directly justifies Stage 2 (ChromaDB RAG Knowledge Store) and our Evaluation Protocol. We adopt Vul-RAG's insight by indexing 969 official NIST CWE definitions and DiverseVul/CVEfixes patch diffs in ChromaDB to eliminate patch-blindness. We strictly adhere to Chasing Shadows by adopting False Discovery Rate (FDR) as our primary metric, achieving FDR = 0.0% on our benchmark suite (eliminating 100% of SAST false alarms).</t>
+          <t>Directly justifies Stage 2 (ChromaDB RAG Knowledge Store) and our Evaluation Protocol. We adopt Vul-RAG's insight by indexing 969 official NIST CWE definitions and DiverseVul/CVEfixes patch diffs in ChromaDB to eliminate patch-blindness. We strictly adhere to Chasing Shadows by adopting False Discovery Rate (FDR) as our primary metric, achieving FDR = 0.0% across our pilot micro-benchmark (resolving all 4 Flawfinder false alarms on the evaluated pairs).</t>
         </is>
       </c>
       <c r="B19" s="11" t="n"/>
@@ -3358,7 +3358,7 @@
     <row r="46" ht="50" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>Alignment with AstraVul: Directly justifies Stage 2 (ChromaDB RAG Knowledge Store) and our Evaluation Protocol. We adopt Vul-RAG's insight by indexing 969 official NIST CWE definitions and DiverseVul/CVEfixes patch diffs in ChromaDB to eliminate patch-blindness. We strictly adhere to Chasing Shadows by adopting False Discovery Rate (FDR) as our primary metric, achieving FDR = 0.0% on our benchmark suite (eliminating 100% of SAST false alarms).</t>
+          <t>Alignment with AstraVul: Directly justifies Stage 2 (ChromaDB RAG Knowledge Store) and our Evaluation Protocol. We adopt Vul-RAG's insight by indexing 969 official NIST CWE definitions and DiverseVul/CVEfixes patch diffs in ChromaDB to eliminate patch-blindness. We strictly adhere to Chasing Shadows by adopting False Discovery Rate (FDR) as our primary metric, achieving FDR = 0.0% across our pilot micro-benchmark (resolving all 4 Flawfinder false alarms on the evaluated pairs).</t>
         </is>
       </c>
       <c r="B46" s="11" t="n"/>

</xml_diff>